<commit_message>
Mileage sheet: keep header blank, keep the CTO/SC note, dd-mm-yyyy dates, 21/04 counts as 21/24
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RBmWy4E5CzyXK6x3B7Neyk
</commit_message>
<xml_diff>
--- a/ti-goods-roster/assets/mileage-template.xlsx
+++ b/ti-goods-roster/assets/mileage-template.xlsx
@@ -2033,7 +2033,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X82"/>
+  <dimension ref="B1:S82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="24.140625" customWidth="1" style="129" min="2" max="2"/>
@@ -2056,7 +2056,7 @@
       <c r="B1" s="264" t="inlineStr">
         <is>
           <t xml:space="preserve">STATEMENT OF WORK DONE AND KILOMETERAGE EARNED BY                                                                                                                                                                                                                        RANK:                               BASIC:                             HQtrs -            RATE per 100 kms Rs.                                  STAFF/TKT No.          
-PERIOD START :01/09/2026                                                                                                            ENDING:  30/09/2026                               </t>
+PERIOD START :                                                                                                            ENDING:                               </t>
         </is>
       </c>
       <c r="C1" s="265" t="n"/>
@@ -2231,7 +2231,11 @@
       <c r="D5" s="145" t="n"/>
       <c r="E5" s="145" t="n"/>
       <c r="F5" s="116" t="n"/>
-      <c r="G5" s="274" t="n"/>
+      <c r="G5" s="274" t="inlineStr">
+        <is>
+          <t>WORKING IN CTO/SC</t>
+        </is>
+      </c>
       <c r="H5" s="275" t="n"/>
       <c r="I5" s="275" t="n"/>
       <c r="J5" s="275" t="n"/>
@@ -3172,37 +3176,6 @@
       <c r="R49" s="45" t="n"/>
       <c r="S49" s="46" t="n"/>
     </row>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
     <row r="81">
       <c r="O81" s="11" t="n"/>
       <c r="P81" s="11" t="n"/>

</xml_diff>